<commit_message>
📊 V9.2.1 daily run 2026-05-18_05:38
</commit_message>
<xml_diff>
--- a/paper_trades/dashboard_2026-05-18.xlsx
+++ b/paper_trades/dashboard_2026-05-18.xlsx
@@ -648,17 +648,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -668,64 +668,64 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>32.56</v>
+        <v>15.33</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>30.88</v>
+        <v>14.54</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>34.52</v>
+        <v>16.61</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>36.04</v>
+        <v>17.6</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>12.52</v>
+        <v>9.57</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
         <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>32.9</v>
+        <v>15.84</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>1.04</v>
+        <v>3.33</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>6.63</v>
+        <v>6.33</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-0.12</v>
+        <v>-0.33</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -739,39 +739,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>15.33</v>
+        <v>128.16</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>14.54</v>
+        <v>121.51</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>16.61</v>
+        <v>135.22</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>17.6</v>
+        <v>140.71</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>9.57</v>
+        <v>5.12</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>15.84</v>
+        <v>128.9</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>3.33</v>
+        <v>0.58</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>6.33</v>
+        <v>1.12</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-0.33</v>
+        <v>-1.69</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>128.16</v>
+        <v>14.64</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>121.51</v>
+        <v>13.88</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>135.22</v>
+        <v>15.47</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>140.71</v>
+        <v>16.12</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>5.12</v>
+        <v>3.78</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>128.9</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>0.58</v>
+        <v>14.25</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>-2.66</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>1.12</v>
+        <v>0.55</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-1.69</v>
+        <v>-3.21</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -869,43 +869,43 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>14.64</v>
+        <v>158.92</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>13.88</v>
+        <v>150.69</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>15.47</v>
+        <v>166.51</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>16.12</v>
+        <v>172.44</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3.78</v>
+        <v>3.46</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>14.25</v>
+        <v>154.1</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>-2.66</v>
+        <v>-3.03</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-3.21</v>
+        <v>-3.41</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,22 +916,22 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -940,39 +940,39 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>158.92</v>
+        <v>14.6</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>150.69</v>
+        <v>13.84</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>166.51</v>
+        <v>15.39</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>172.44</v>
+        <v>16.01</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>3.46</v>
+        <v>3.63</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>154.1</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>-3.03</v>
+        <v>14.95</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>2.4</v>
       </c>
       <c r="O8" s="8" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="P8" s="8" t="n">
         <v>0</v>
-      </c>
-      <c r="P8" s="8" t="n">
-        <v>-3.41</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -993,53 +993,53 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>14.6</v>
+        <v>28.94</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>13.84</v>
+        <v>27.44</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>15.39</v>
+        <v>30.84</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>16.01</v>
+        <v>32.3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3.63</v>
+        <v>3</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>14.95</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>2.4</v>
+        <v>28.6</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>-1.17</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>4.45</v>
+        <v>0.48</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0</v>
+        <v>-2.28</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,63 +1050,63 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>28.94</v>
+        <v>11.35</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>27.44</v>
+        <v>10.76</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>30.84</v>
+        <v>12.01</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>32.3</v>
+        <v>12.51</v>
       </c>
       <c r="J10" s="6" t="n">
+        <v>16.05</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="O10" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>7%</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>-1.17</v>
-      </c>
-      <c r="O10" s="8" t="n">
-        <v>0.48</v>
-      </c>
       <c r="P10" s="8" t="n">
-        <v>-2.28</v>
+        <v>-3.44</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1141,39 +1141,39 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>11.82</v>
+        <v>230.06</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>11.21</v>
+        <v>220.32</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>12.43</v>
+        <v>238.88</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>12.91</v>
+        <v>245.84</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>16.94</v>
+        <v>12.77</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>11.82</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>0</v>
+        <v>229.6</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>-0.2</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0</v>
+        <v>-2.03</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1184,7 +1184,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1194,44 +1194,44 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>11.35</v>
+        <v>11.03</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>10.76</v>
+        <v>10.47</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>12.01</v>
+        <v>11.58</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>12.51</v>
+        <v>12.15</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>16.05</v>
+        <v>10.8</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>11.35</v>
+        <v>11.03</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1251,7 +1251,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1261,44 +1261,44 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>230.06</v>
+        <v>32.97</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>220.32</v>
+        <v>31.39</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>238.88</v>
+        <v>34.55</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>245.84</v>
+        <v>36.13</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>12.77</v>
+        <v>7.94</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>230.06</v>
+        <v>32.97</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1560,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1589,64 +1589,64 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>43.14</v>
+        <v>32.9</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0</v>
+        <v>0.0663</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0012</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>12.84</v>
+        <v>12.52</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1655,64 +1655,64 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>12.24</v>
+        <v>11.82</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>12.9</v>
+        <v>11.15</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>1</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0728</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>16.08</v>
+        <v>16.94</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>36.7</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1721,44 +1721,44 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>25.85</v>
+        <v>45.31</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>25.22</v>
+        <v>43.14</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.0244</v>
+        <v>-0.0478</v>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0461</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.35</v>
+        <v>12.84</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>26.1</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1773,12 +1773,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1787,16 +1787,16 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>90.63</v>
+        <v>12.24</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>12.9</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.0416</v>
+        <v>0.0609</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
@@ -1809,22 +1809,22 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.057</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>14.18</v>
+        <v>16.08</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>23</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1853,20 +1853,20 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>15.53</v>
+        <v>25.85</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>15.88</v>
+        <v>25.22</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+      <c r="J10" s="9" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -1875,22 +1875,22 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>0</v>
+        <v>-0.0352</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>11.78</v>
+        <v>14.35</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>19.9</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1905,12 +1905,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1919,20 +1919,20 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>694.39</v>
+        <v>90.63</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>680</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J11" s="9" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J11" s="7" t="n">
+        <v>0.0416</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1941,42 +1941,42 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.057</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0517</v>
+        <v>0</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.02</v>
+        <v>14.18</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>23.7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1985,20 +1985,20 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>15.01</v>
+        <v>15.53</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>14.34</v>
+        <v>15.88</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="9" t="n">
-        <v>-0.0446</v>
-      </c>
-      <c r="K12" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J12" s="7" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -2007,60 +2007,60 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.038</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O12" s="6" t="n">
         <v>11.78</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>11.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>28.9</v>
+        <v>694.39</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>28.16</v>
+        <v>680</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>-0.0256</v>
+        <v>-0.0207</v>
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
@@ -2073,42 +2073,42 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0</v>
+        <v>0.0254</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0517</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>12.9</v>
+        <v>10.02</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>32.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2117,16 +2117,16 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>70.64</v>
+        <v>15.01</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>69</v>
+        <v>14.34</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>-0.0232</v>
+        <v>-0.0446</v>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
@@ -2139,93 +2139,93 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0127</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0466</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>13.3</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>182.46</v>
+        <v>28.9</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>198.78</v>
+        <v>28.16</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+        <v>3</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0436</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>23.45</v>
+        <v>12.9</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>12.1</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2235,63 +2235,63 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>14.05</v>
+        <v>70.64</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>13.25</v>
+        <v>69</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>-0.0567</v>
+        <v>-0.0232</v>
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0178</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0331</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>14.88</v>
+        <v>24.18</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>35.5</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -2301,96 +2301,96 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>14.51</v>
+        <v>198.78</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J17" s="9" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.106</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0036</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>20.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>32.56</v>
+        <v>14.05</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>30.73</v>
+        <v>13.25</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0567</v>
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
@@ -2403,88 +2403,88 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0036</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.079</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>15.98</v>
+        <v>14.88</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>43.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0089</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>13.05</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2499,12 +2499,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2513,16 +2513,16 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0563</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -2535,22 +2535,22 @@
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>12.93</v>
+        <v>15.98</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2565,12 +2565,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2579,16 +2579,16 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0478</v>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
@@ -2601,37 +2601,37 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>12.53</v>
+        <v>13.05</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2645,64 +2645,64 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>-0.0478</v>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>32.16</v>
+        <v>12.93</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,44 +2711,44 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J23" s="7" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K23" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>30.86</v>
+        <v>12.53</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2777,16 +2777,16 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>27.31</v>
+        <v>43.19</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>27.86</v>
+        <v>43.88</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>0.0201</v>
+        <v>0.016</v>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
@@ -2799,22 +2799,22 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0188</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0016</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>26.27</v>
+        <v>32.16</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>23.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2843,16 +2843,16 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>37.25</v>
+        <v>137.37</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>38.14</v>
+        <v>143</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0239</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
@@ -2865,22 +2865,22 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0432</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.002</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>23.8</v>
+        <v>30.86</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>27.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2895,12 +2895,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2909,20 +2909,20 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>105.01</v>
+        <v>27.31</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>105</v>
+        <v>27.86</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="9" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K26" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J26" s="7" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2931,22 +2931,22 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0392</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0114</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>10.01</v>
+        <v>26.27</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>17.6</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2956,39 +2956,39 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>26.25</v>
+        <v>37.25</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>25.64</v>
+        <v>38.14</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J27" s="9" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K27" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -2997,22 +2997,22 @@
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0379</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0212</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>16.26</v>
+        <v>23.8</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3022,39 +3022,39 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>10.7</v>
+        <v>105.01</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>10.73</v>
+        <v>105</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J28" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K28" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>5</v>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -3063,22 +3063,22 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0075</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.022</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>12.8</v>
+        <v>10.01</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3088,122 +3088,254 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>-0.0568</v>
+        <v>-0.0232</v>
       </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K30" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M30" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N30" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P30" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O31" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P31" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="G32" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H32" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="9" t="n">
+      <c r="I32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K30" s="10" t="inlineStr">
+      <c r="K32" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M30" s="8" t="n">
+      <c r="M32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="8" t="n">
+      <c r="N32" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O30" s="6" t="n">
+      <c r="O32" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P30" s="6" t="n">
+      <c r="P32" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3221,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3238,7 +3370,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-18T02:02:30</t>
+          <t>محسوب في: 2026-05-18T05:38:00</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3394,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -3282,7 +3414,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -3292,7 +3424,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -3303,7 +3435,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>34.5%</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3459,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.74%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3470,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="13">
@@ -3349,7 +3481,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-35.04%</t>
+          <t>-37.14%</t>
         </is>
       </c>
     </row>
@@ -3483,19 +3615,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.49%</t>
         </is>
       </c>
     </row>
@@ -3589,19 +3721,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>-3.23%</t>
         </is>
       </c>
     </row>
@@ -3635,19 +3767,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>+0.48%</t>
+          <t>-0.74%</t>
         </is>
       </c>
     </row>
@@ -3848,6 +3980,13 @@
     <row r="50"/>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
+        <is>
+          <t>2370: 1/3 = 33.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>2280: 0/3 = 0.0%</t>
         </is>
@@ -3868,7 +4007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4302,53 +4441,53 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>2</v>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-2.58%</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+3.53%</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -4367,29 +4506,29 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -4408,29 +4547,29 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -4449,29 +4588,29 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -4490,29 +4629,29 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -4531,29 +4670,29 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -4572,39 +4711,39 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
@@ -4613,17 +4752,17 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-0.89%</t>
         </is>
       </c>
     </row>
@@ -4911,6 +5050,47 @@
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>-5.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>8070</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>

</xml_diff>